<commit_message>
Updates for wiring layout builder
</commit_message>
<xml_diff>
--- a/pathfinder/Papaya Wiring Layout.xlsx
+++ b/pathfinder/Papaya Wiring Layout.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d0c8f507161f927/CodingProjects/papaya-pathfinder/pathfinder/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LocalRepos\papaya-pathfinder\pathfinder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="566" documentId="8_{F67DEC02-DD7F-469A-89B3-826B41FA7950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34011E39-F523-4852-BF7C-50E60D7136AF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE644C35-734C-47BB-B0A8-F7818AFCFBCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F4C2A71C-EFB8-4AB8-A324-8B57417C3AED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F4C2A71C-EFB8-4AB8-A324-8B57417C3AED}"/>
   </bookViews>
   <sheets>
-    <sheet name="Wiring Layout" sheetId="1" r:id="rId1"/>
+    <sheet name="Wiring Layout v2" sheetId="2" r:id="rId1"/>
+    <sheet name="Wiring Layout" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="250">
   <si>
     <t>A</t>
   </si>
@@ -2177,34 +2177,91 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2225,79 +2282,22 @@
     <xf numFmtId="0" fontId="1" fillId="11" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2318,6 +2318,440 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>297656</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>39687</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>456406</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>39687</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="2" name="Straight Arrow Connector 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{37D9BB44-EFF1-44B2-9334-1EF6C96A2458}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="12975431" y="677862"/>
+          <a:ext cx="1835150" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:prstDash val="dash"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>198444</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>188516</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>208366</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>119063</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="3" name="Straight Arrow Connector 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D95121D4-F197-4DDE-B2A2-CD9E1C3E0F72}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16124244" y="1026716"/>
+          <a:ext cx="9922" cy="1445022"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:prstDash val="dash"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>486172</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>29765</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>138906</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="Rectangle 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5A819325-CC28-E904-F686-2E09A9FE7498}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1091406" y="5208984"/>
+          <a:ext cx="2401094" cy="1279922"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2400"/>
+            <a:t>No</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>112711</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>182165</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>347264</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>192087</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="Rectangle 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E0557A47-9B49-82A7-463C-F456E08608A3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2980133" y="817165"/>
+          <a:ext cx="7556897" cy="1279922"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2400"/>
+            <a:t>No</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>251618</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>202009</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>3571</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>172244</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="Rectangle 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72E94A25-2955-88E4-A5BE-A27852A36D4A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12465446" y="5162947"/>
+          <a:ext cx="2401094" cy="1279922"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2400"/>
+            <a:t>No</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>43</xdr:col>
+      <xdr:colOff>86518</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>215502</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>47</xdr:col>
+      <xdr:colOff>66674</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>185737</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="Rectangle 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8D98F090-70C2-6BBC-7546-A853797BEEA7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="23899018" y="5176440"/>
+          <a:ext cx="2401094" cy="1279922"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2400"/>
+            <a:t>No</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>334564</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>215504</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>9922</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>208360</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="Rectangle 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1166021B-88D5-BD4A-28FC-A94936FA8E06}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11060111" y="1247379"/>
+          <a:ext cx="677467" cy="647700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2400"/>
+            <a:t>No</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -2434,10 +2868,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2756,14 +3186,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{639F2336-69B3-4605-B191-23BB70925903}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D60F6980-CF43-4E73-90A6-31EF4328F7B8}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AD52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="155"/>
+    <col min="1" max="1" width="9.140625" style="118"/>
     <col min="3" max="3" width="7.28515625" customWidth="1"/>
     <col min="4" max="4" width="8.42578125" customWidth="1"/>
     <col min="5" max="5" width="9.140625" customWidth="1"/>
@@ -2811,13 +3241,13 @@
       <c r="X1" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="Y1" s="143" t="s">
+      <c r="Y1" s="131" t="s">
         <v>65</v>
       </c>
-      <c r="Z1" s="143"/>
-      <c r="AA1" s="143"/>
-      <c r="AB1" s="143"/>
-      <c r="AC1" s="143"/>
+      <c r="Z1" s="131"/>
+      <c r="AA1" s="131"/>
+      <c r="AB1" s="131"/>
+      <c r="AC1" s="131"/>
     </row>
     <row r="2" spans="1:30" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D2" s="62" t="s">
@@ -2844,11 +3274,11 @@
       <c r="X2" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="Y2" s="143"/>
-      <c r="Z2" s="143"/>
-      <c r="AA2" s="143"/>
-      <c r="AB2" s="143"/>
-      <c r="AC2" s="143"/>
+      <c r="Y2" s="131"/>
+      <c r="Z2" s="131"/>
+      <c r="AA2" s="131"/>
+      <c r="AB2" s="131"/>
+      <c r="AC2" s="131"/>
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="E3" s="63" t="s">
@@ -2940,7 +3370,7 @@
       </c>
     </row>
     <row r="6" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="156" t="s">
+      <c r="A6" s="119" t="s">
         <v>30</v>
       </c>
       <c r="B6" s="22" t="s">
@@ -2952,11 +3382,11 @@
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="16"/>
-      <c r="G6" s="137" t="s">
+      <c r="G6" s="133" t="s">
         <v>94</v>
       </c>
-      <c r="H6" s="138"/>
-      <c r="I6" s="139"/>
+      <c r="H6" s="134"/>
+      <c r="I6" s="135"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1" t="s">
         <v>248</v>
@@ -2964,12 +3394,12 @@
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
-      <c r="O6" s="137" t="s">
+      <c r="O6" s="133" t="s">
         <v>94</v>
       </c>
-      <c r="P6" s="138"/>
-      <c r="Q6" s="138"/>
-      <c r="R6" s="139"/>
+      <c r="P6" s="134"/>
+      <c r="Q6" s="134"/>
+      <c r="R6" s="135"/>
       <c r="S6" s="64" t="s">
         <v>49</v>
       </c>
@@ -2977,26 +3407,26 @@
       <c r="U6" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="V6" s="148" t="s">
+      <c r="V6" s="136" t="s">
         <v>94</v>
       </c>
-      <c r="W6" s="148"/>
-      <c r="X6" s="148"/>
-      <c r="Y6" s="148"/>
-      <c r="Z6" s="148"/>
-      <c r="AA6" s="148"/>
+      <c r="W6" s="136"/>
+      <c r="X6" s="136"/>
+      <c r="Y6" s="136"/>
+      <c r="Z6" s="136"/>
+      <c r="AA6" s="136"/>
       <c r="AB6" s="9" t="s">
         <v>89</v>
       </c>
       <c r="AC6" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="AD6" s="156" t="s">
+      <c r="AD6" s="119" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="157" t="s">
+      <c r="A7" s="120" t="s">
         <v>29</v>
       </c>
       <c r="B7" s="22" t="s">
@@ -3065,12 +3495,12 @@
       <c r="AC7" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="AD7" s="157" t="s">
+      <c r="AD7" s="120" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="157" t="s">
+      <c r="A8" s="120" t="s">
         <v>28</v>
       </c>
       <c r="B8" s="22" t="s">
@@ -3113,24 +3543,24 @@
       </c>
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
-      <c r="V8" s="145" t="s">
+      <c r="V8" s="122" t="s">
         <v>38</v>
       </c>
-      <c r="W8" s="146"/>
-      <c r="X8" s="146"/>
-      <c r="Y8" s="146"/>
-      <c r="Z8" s="146"/>
-      <c r="AA8" s="147"/>
+      <c r="W8" s="123"/>
+      <c r="X8" s="123"/>
+      <c r="Y8" s="123"/>
+      <c r="Z8" s="123"/>
+      <c r="AA8" s="124"/>
       <c r="AB8" s="1"/>
       <c r="AC8" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="AD8" s="157" t="s">
+      <c r="AD8" s="120" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="157" t="s">
+      <c r="A9" s="120" t="s">
         <v>27</v>
       </c>
       <c r="B9" s="22" t="s">
@@ -3140,22 +3570,22 @@
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
-      <c r="G9" s="134" t="s">
+      <c r="G9" s="128" t="s">
         <v>94</v>
       </c>
-      <c r="H9" s="135"/>
-      <c r="I9" s="136"/>
+      <c r="H9" s="129"/>
+      <c r="I9" s="130"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
-      <c r="O9" s="134" t="s">
+      <c r="O9" s="128" t="s">
         <v>94</v>
       </c>
-      <c r="P9" s="135"/>
-      <c r="Q9" s="135"/>
-      <c r="R9" s="136"/>
+      <c r="P9" s="129"/>
+      <c r="Q9" s="129"/>
+      <c r="R9" s="130"/>
       <c r="S9" s="1"/>
       <c r="T9" s="1"/>
       <c r="U9" s="1"/>
@@ -3169,12 +3599,12 @@
       <c r="AC9" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="AD9" s="157" t="s">
+      <c r="AD9" s="120" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="157" t="s">
+      <c r="A10" s="120" t="s">
         <v>26</v>
       </c>
       <c r="B10" s="22" t="s">
@@ -3184,22 +3614,22 @@
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
-      <c r="G10" s="145" t="s">
+      <c r="G10" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="H10" s="146"/>
-      <c r="I10" s="147"/>
+      <c r="H10" s="123"/>
+      <c r="I10" s="124"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
-      <c r="O10" s="145" t="s">
+      <c r="O10" s="122" t="s">
         <v>48</v>
       </c>
-      <c r="P10" s="146"/>
-      <c r="Q10" s="146"/>
-      <c r="R10" s="147"/>
+      <c r="P10" s="123"/>
+      <c r="Q10" s="123"/>
+      <c r="R10" s="124"/>
       <c r="S10" s="1"/>
       <c r="T10" s="1"/>
       <c r="U10" s="1"/>
@@ -3213,24 +3643,24 @@
       <c r="AC10" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="AD10" s="157" t="s">
+      <c r="AD10" s="120" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="157" t="s">
+      <c r="A11" s="120" t="s">
         <v>25</v>
       </c>
       <c r="B11" s="22" t="s">
         <v>5</v>
       </c>
       <c r="C11" s="1"/>
-      <c r="D11" s="137" t="s">
+      <c r="D11" s="133" t="s">
         <v>94</v>
       </c>
-      <c r="E11" s="138"/>
-      <c r="F11" s="138"/>
-      <c r="G11" s="139"/>
+      <c r="E11" s="134"/>
+      <c r="F11" s="134"/>
+      <c r="G11" s="135"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
@@ -3247,22 +3677,22 @@
       <c r="U11" s="2"/>
       <c r="V11" s="1"/>
       <c r="W11" s="1"/>
-      <c r="X11" s="137" t="s">
+      <c r="X11" s="133" t="s">
         <v>94</v>
       </c>
-      <c r="Y11" s="138"/>
-      <c r="Z11" s="138"/>
-      <c r="AA11" s="139"/>
+      <c r="Y11" s="134"/>
+      <c r="Z11" s="134"/>
+      <c r="AA11" s="135"/>
       <c r="AB11" s="1"/>
       <c r="AC11" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="AD11" s="157" t="s">
+      <c r="AD11" s="120" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="157" t="s">
+      <c r="A12" s="120" t="s">
         <v>24</v>
       </c>
       <c r="B12" s="22" t="s">
@@ -3285,17 +3715,17 @@
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
       <c r="K12" s="4"/>
-      <c r="L12" s="149" t="s">
+      <c r="L12" s="137" t="s">
         <v>31</v>
       </c>
-      <c r="M12" s="150"/>
-      <c r="N12" s="150"/>
-      <c r="O12" s="150"/>
-      <c r="P12" s="150"/>
-      <c r="Q12" s="150"/>
-      <c r="R12" s="150"/>
-      <c r="S12" s="150"/>
-      <c r="T12" s="151"/>
+      <c r="M12" s="138"/>
+      <c r="N12" s="138"/>
+      <c r="O12" s="138"/>
+      <c r="P12" s="138"/>
+      <c r="Q12" s="138"/>
+      <c r="R12" s="138"/>
+      <c r="S12" s="138"/>
+      <c r="T12" s="139"/>
       <c r="U12" s="5"/>
       <c r="V12" s="1"/>
       <c r="W12" s="1"/>
@@ -3315,24 +3745,24 @@
       <c r="AC12" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="AD12" s="157" t="s">
+      <c r="AD12" s="120" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="157" t="s">
+      <c r="A13" s="120" t="s">
         <v>23</v>
       </c>
       <c r="B13" s="22" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="1"/>
-      <c r="D13" s="145" t="s">
+      <c r="D13" s="122" t="s">
         <v>58</v>
       </c>
-      <c r="E13" s="146"/>
-      <c r="F13" s="146"/>
-      <c r="G13" s="147"/>
+      <c r="E13" s="123"/>
+      <c r="F13" s="123"/>
+      <c r="G13" s="124"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
@@ -3353,34 +3783,34 @@
       </c>
       <c r="V13" s="1"/>
       <c r="W13" s="1"/>
-      <c r="X13" s="145" t="s">
+      <c r="X13" s="122" t="s">
         <v>60</v>
       </c>
-      <c r="Y13" s="146"/>
-      <c r="Z13" s="146"/>
-      <c r="AA13" s="147"/>
+      <c r="Y13" s="123"/>
+      <c r="Z13" s="123"/>
+      <c r="AA13" s="124"/>
       <c r="AB13" s="1"/>
       <c r="AC13" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="AD13" s="157" t="s">
+      <c r="AD13" s="120" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="157" t="s">
+      <c r="A14" s="120" t="s">
         <v>22</v>
       </c>
       <c r="B14" s="22" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="1"/>
-      <c r="D14" s="137" t="s">
+      <c r="D14" s="133" t="s">
         <v>94</v>
       </c>
-      <c r="E14" s="138"/>
-      <c r="F14" s="138"/>
-      <c r="G14" s="139"/>
+      <c r="E14" s="134"/>
+      <c r="F14" s="134"/>
+      <c r="G14" s="135"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="7"/>
@@ -3411,12 +3841,12 @@
       <c r="AC14" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="AD14" s="157" t="s">
+      <c r="AD14" s="120" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="157" t="s">
+      <c r="A15" s="120" t="s">
         <v>21</v>
       </c>
       <c r="B15" s="22" t="s">
@@ -3456,23 +3886,23 @@
       </c>
       <c r="U15" s="100"/>
       <c r="V15" s="9"/>
-      <c r="W15" s="137" t="s">
+      <c r="W15" s="133" t="s">
         <v>94</v>
       </c>
-      <c r="X15" s="138"/>
-      <c r="Y15" s="138"/>
-      <c r="Z15" s="138"/>
-      <c r="AA15" s="139"/>
+      <c r="X15" s="134"/>
+      <c r="Y15" s="134"/>
+      <c r="Z15" s="134"/>
+      <c r="AA15" s="135"/>
       <c r="AB15" s="1"/>
       <c r="AC15" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="AD15" s="157" t="s">
+      <c r="AD15" s="120" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="157" t="s">
+      <c r="A16" s="120" t="s">
         <v>20</v>
       </c>
       <c r="B16" s="22" t="s">
@@ -3533,23 +3963,23 @@
       <c r="AC16" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="AD16" s="157" t="s">
+      <c r="AD16" s="120" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="157" t="s">
+      <c r="A17" s="120" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="22" t="s">
         <v>11</v>
       </c>
       <c r="C17" s="1"/>
-      <c r="D17" s="140" t="s">
+      <c r="D17" s="125" t="s">
         <v>94</v>
       </c>
-      <c r="E17" s="141"/>
-      <c r="F17" s="142"/>
+      <c r="E17" s="126"/>
+      <c r="F17" s="127"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="7"/>
@@ -3590,12 +4020,12 @@
       <c r="AC17" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="AD17" s="157" t="s">
+      <c r="AD17" s="120" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="157" t="s">
+      <c r="A18" s="120" t="s">
         <v>18</v>
       </c>
       <c r="B18" s="22" t="s">
@@ -3625,23 +4055,23 @@
       </c>
       <c r="U18" s="100"/>
       <c r="V18" s="9"/>
-      <c r="W18" s="134" t="s">
+      <c r="W18" s="128" t="s">
         <v>94</v>
       </c>
-      <c r="X18" s="135"/>
-      <c r="Y18" s="135"/>
-      <c r="Z18" s="135"/>
-      <c r="AA18" s="136"/>
+      <c r="X18" s="129"/>
+      <c r="Y18" s="129"/>
+      <c r="Z18" s="129"/>
+      <c r="AA18" s="130"/>
       <c r="AB18" s="1"/>
       <c r="AC18" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="AD18" s="157" t="s">
+      <c r="AD18" s="120" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="157" t="s">
+      <c r="A19" s="120" t="s">
         <v>17</v>
       </c>
       <c r="B19" s="22" t="s">
@@ -3685,23 +4115,23 @@
       <c r="V19" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="W19" s="145" t="s">
+      <c r="W19" s="122" t="s">
         <v>61</v>
       </c>
-      <c r="X19" s="146"/>
-      <c r="Y19" s="146"/>
-      <c r="Z19" s="146"/>
-      <c r="AA19" s="147"/>
+      <c r="X19" s="123"/>
+      <c r="Y19" s="123"/>
+      <c r="Z19" s="123"/>
+      <c r="AA19" s="124"/>
       <c r="AB19" s="1"/>
       <c r="AC19" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="AD19" s="157" t="s">
+      <c r="AD19" s="120" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="157" t="s">
+      <c r="A20" s="120" t="s">
         <v>16</v>
       </c>
       <c r="B20" s="22" t="s">
@@ -3711,10 +4141,10 @@
       <c r="D20" s="1"/>
       <c r="E20" s="7"/>
       <c r="F20" s="113"/>
-      <c r="G20" s="152" t="s">
+      <c r="G20" s="140" t="s">
         <v>50</v>
       </c>
-      <c r="H20" s="152"/>
+      <c r="H20" s="140"/>
       <c r="I20" s="114"/>
       <c r="J20" s="24" t="s">
         <v>201</v>
@@ -3754,12 +4184,12 @@
       <c r="AC20" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="AD20" s="157" t="s">
+      <c r="AD20" s="120" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="157" t="s">
+      <c r="A21" s="120" t="s">
         <v>15</v>
       </c>
       <c r="B21" s="22" t="s">
@@ -3773,8 +4203,8 @@
       </c>
       <c r="E21" s="7"/>
       <c r="F21" s="113"/>
-      <c r="G21" s="153"/>
-      <c r="H21" s="153"/>
+      <c r="G21" s="141"/>
+      <c r="H21" s="141"/>
       <c r="I21" s="114"/>
       <c r="J21" s="24"/>
       <c r="K21" s="70"/>
@@ -3806,12 +4236,12 @@
       <c r="AC21" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="AD21" s="157" t="s">
+      <c r="AD21" s="120" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="157" t="s">
+      <c r="A22" s="120" t="s">
         <v>14</v>
       </c>
       <c r="B22" s="22" t="s">
@@ -3825,8 +4255,8 @@
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="113"/>
-      <c r="G22" s="153"/>
-      <c r="H22" s="153"/>
+      <c r="G22" s="141"/>
+      <c r="H22" s="141"/>
       <c r="I22" s="114"/>
       <c r="J22" s="24"/>
       <c r="K22" s="70"/>
@@ -3858,12 +4288,12 @@
       <c r="AC22" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="AD22" s="157" t="s">
+      <c r="AD22" s="120" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="157" t="s">
+      <c r="A23" s="120" t="s">
         <v>13</v>
       </c>
       <c r="B23" s="22" t="s">
@@ -3877,8 +4307,8 @@
       </c>
       <c r="E23" s="7"/>
       <c r="F23" s="113"/>
-      <c r="G23" s="154"/>
-      <c r="H23" s="154"/>
+      <c r="G23" s="142"/>
+      <c r="H23" s="142"/>
       <c r="I23" s="114"/>
       <c r="J23" s="24"/>
       <c r="K23" s="70"/>
@@ -3918,12 +4348,12 @@
       <c r="AC23" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="AD23" s="157" t="s">
+      <c r="AD23" s="120" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="157" t="s">
+      <c r="A24" s="120" t="s">
         <v>12</v>
       </c>
       <c r="B24" s="22" t="s">
@@ -3974,12 +4404,12 @@
       <c r="AC24" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="AD24" s="157" t="s">
+      <c r="AD24" s="120" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="25" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="157" t="s">
+      <c r="A25" s="120" t="s">
         <v>11</v>
       </c>
       <c r="B25" s="22" t="s">
@@ -4026,18 +4456,18 @@
       <c r="AC25" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="AD25" s="157" t="s">
+      <c r="AD25" s="120" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="26" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="157" t="s">
+      <c r="A26" s="120" t="s">
         <v>10</v>
       </c>
       <c r="B26" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="128" t="s">
+      <c r="C26" s="147" t="s">
         <v>94</v>
       </c>
       <c r="D26" s="87" t="s">
@@ -4046,7 +4476,7 @@
       <c r="E26" s="88" t="s">
         <v>168</v>
       </c>
-      <c r="F26" s="131" t="s">
+      <c r="F26" s="150" t="s">
         <v>94</v>
       </c>
       <c r="G26" s="1"/>
@@ -4071,7 +4501,7 @@
       <c r="V26" s="9"/>
       <c r="W26" s="1"/>
       <c r="X26" s="1"/>
-      <c r="Y26" s="128" t="s">
+      <c r="Y26" s="147" t="s">
         <v>94</v>
       </c>
       <c r="Z26" s="87" t="s">
@@ -4080,31 +4510,31 @@
       <c r="AA26" s="88" t="s">
         <v>171</v>
       </c>
-      <c r="AB26" s="131" t="s">
+      <c r="AB26" s="150" t="s">
         <v>94</v>
       </c>
       <c r="AC26" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="AD26" s="157" t="s">
+      <c r="AD26" s="120" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="157" t="s">
+      <c r="A27" s="120" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="129"/>
+      <c r="C27" s="148"/>
       <c r="D27" s="89" t="s">
         <v>190</v>
       </c>
       <c r="E27" s="90" t="s">
         <v>189</v>
       </c>
-      <c r="F27" s="132"/>
+      <c r="F27" s="151"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
@@ -4127,36 +4557,36 @@
       <c r="V27" s="9"/>
       <c r="W27" s="1"/>
       <c r="X27" s="1"/>
-      <c r="Y27" s="129"/>
+      <c r="Y27" s="148"/>
       <c r="Z27" s="89" t="s">
         <v>230</v>
       </c>
       <c r="AA27" s="90" t="s">
         <v>231</v>
       </c>
-      <c r="AB27" s="132"/>
+      <c r="AB27" s="151"/>
       <c r="AC27" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="AD27" s="157" t="s">
+      <c r="AD27" s="120" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="157" t="s">
+      <c r="A28" s="120" t="s">
         <v>8</v>
       </c>
       <c r="B28" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="C28" s="129"/>
+      <c r="C28" s="148"/>
       <c r="D28" s="89" t="s">
         <v>191</v>
       </c>
       <c r="E28" s="90" t="s">
         <v>188</v>
       </c>
-      <c r="F28" s="132"/>
+      <c r="F28" s="151"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
@@ -4179,36 +4609,36 @@
       <c r="V28" s="9"/>
       <c r="W28" s="1"/>
       <c r="X28" s="1"/>
-      <c r="Y28" s="129"/>
+      <c r="Y28" s="148"/>
       <c r="Z28" s="89" t="s">
         <v>229</v>
       </c>
       <c r="AA28" s="90" t="s">
         <v>232</v>
       </c>
-      <c r="AB28" s="132"/>
+      <c r="AB28" s="151"/>
       <c r="AC28" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="AD28" s="157" t="s">
+      <c r="AD28" s="120" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="157" t="s">
+      <c r="A29" s="120" t="s">
         <v>7</v>
       </c>
       <c r="B29" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="C29" s="130"/>
+      <c r="C29" s="149"/>
       <c r="D29" s="91" t="s">
         <v>186</v>
       </c>
       <c r="E29" s="92" t="s">
         <v>187</v>
       </c>
-      <c r="F29" s="133"/>
+      <c r="F29" s="152"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
@@ -4235,23 +4665,23 @@
       <c r="V29" s="9"/>
       <c r="W29" s="1"/>
       <c r="X29" s="1"/>
-      <c r="Y29" s="130"/>
+      <c r="Y29" s="149"/>
       <c r="Z29" s="91" t="s">
         <v>228</v>
       </c>
       <c r="AA29" s="92" t="s">
         <v>233</v>
       </c>
-      <c r="AB29" s="133"/>
+      <c r="AB29" s="152"/>
       <c r="AC29" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="AD29" s="157" t="s">
+      <c r="AD29" s="120" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="30" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="157" t="s">
+      <c r="A30" s="120" t="s">
         <v>6</v>
       </c>
       <c r="B30" s="22" t="s">
@@ -4298,12 +4728,12 @@
       <c r="AC30" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="AD30" s="157" t="s">
+      <c r="AD30" s="120" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="157" t="s">
+      <c r="A31" s="120" t="s">
         <v>5</v>
       </c>
       <c r="B31" s="22" t="s">
@@ -4346,12 +4776,12 @@
       <c r="AC31" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="AD31" s="157" t="s">
+      <c r="AD31" s="120" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="157" t="s">
+      <c r="A32" s="120" t="s">
         <v>4</v>
       </c>
       <c r="B32" s="22" t="s">
@@ -4402,12 +4832,12 @@
       <c r="AC32" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="AD32" s="157" t="s">
+      <c r="AD32" s="120" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="157" t="s">
+      <c r="A33" s="120" t="s">
         <v>3</v>
       </c>
       <c r="B33" s="22" t="s">
@@ -4454,12 +4884,12 @@
       <c r="AC33" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="AD33" s="157" t="s">
+      <c r="AD33" s="120" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="157" t="s">
+      <c r="A34" s="120" t="s">
         <v>2</v>
       </c>
       <c r="B34" s="22" t="s">
@@ -4508,12 +4938,12 @@
       <c r="AC34" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="AD34" s="157" t="s">
+      <c r="AD34" s="120" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="157" t="s">
+      <c r="A35" s="120" t="s">
         <v>1</v>
       </c>
       <c r="B35" s="22" t="s">
@@ -4558,12 +4988,12 @@
       <c r="AC35" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="AD35" s="157" t="s">
+      <c r="AD35" s="120" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="158" t="s">
+      <c r="A36" s="121" t="s">
         <v>0</v>
       </c>
       <c r="B36" s="22" t="s">
@@ -4606,7 +5036,7 @@
       <c r="AC36" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="AD36" s="158" t="s">
+      <c r="AD36" s="121" t="s">
         <v>0</v>
       </c>
     </row>
@@ -4951,47 +5381,47 @@
       <c r="AB46" s="47"/>
     </row>
     <row r="47" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="B47" s="144" t="s">
+      <c r="B47" s="132" t="s">
         <v>79</v>
       </c>
-      <c r="C47" s="144"/>
-      <c r="D47" s="144"/>
-      <c r="E47" s="144"/>
-      <c r="F47" s="144"/>
-      <c r="G47" s="144"/>
-      <c r="K47" s="144" t="s">
+      <c r="C47" s="132"/>
+      <c r="D47" s="132"/>
+      <c r="E47" s="132"/>
+      <c r="F47" s="132"/>
+      <c r="G47" s="132"/>
+      <c r="K47" s="132" t="s">
         <v>81</v>
       </c>
-      <c r="L47" s="144"/>
-      <c r="M47" s="144"/>
-      <c r="N47" s="144"/>
-      <c r="W47" s="144" t="s">
+      <c r="L47" s="132"/>
+      <c r="M47" s="132"/>
+      <c r="N47" s="132"/>
+      <c r="W47" s="132" t="s">
         <v>80</v>
       </c>
-      <c r="X47" s="144"/>
-      <c r="Y47" s="144"/>
-      <c r="Z47" s="144"/>
-      <c r="AA47" s="144"/>
-      <c r="AB47" s="144"/>
+      <c r="X47" s="132"/>
+      <c r="Y47" s="132"/>
+      <c r="Z47" s="132"/>
+      <c r="AA47" s="132"/>
+      <c r="AB47" s="132"/>
     </row>
     <row r="48" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="49" spans="2:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K49" s="124" t="s">
+      <c r="K49" s="157" t="s">
         <v>185</v>
       </c>
-      <c r="L49" s="125"/>
-      <c r="N49" s="124" t="s">
+      <c r="L49" s="158"/>
+      <c r="N49" s="157" t="s">
         <v>198</v>
       </c>
-      <c r="O49" s="125"/>
-      <c r="Q49" s="124" t="s">
+      <c r="O49" s="158"/>
+      <c r="Q49" s="157" t="s">
         <v>240</v>
       </c>
-      <c r="R49" s="125"/>
-      <c r="T49" s="124" t="s">
+      <c r="R49" s="158"/>
+      <c r="T49" s="157" t="s">
         <v>241</v>
       </c>
-      <c r="U49" s="125"/>
+      <c r="U49" s="158"/>
     </row>
     <row r="50" spans="2:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B50" s="115" t="s">
@@ -5012,22 +5442,22 @@
       <c r="I50" s="116" t="s">
         <v>57</v>
       </c>
-      <c r="K50" s="118" t="s">
+      <c r="K50" s="153" t="s">
         <v>179</v>
       </c>
-      <c r="L50" s="119"/>
-      <c r="N50" s="118" t="s">
+      <c r="L50" s="154"/>
+      <c r="N50" s="153" t="s">
         <v>179</v>
       </c>
-      <c r="O50" s="119"/>
-      <c r="Q50" s="118" t="s">
+      <c r="O50" s="154"/>
+      <c r="Q50" s="153" t="s">
         <v>179</v>
       </c>
-      <c r="R50" s="119"/>
-      <c r="T50" s="118" t="s">
+      <c r="R50" s="154"/>
+      <c r="T50" s="153" t="s">
         <v>179</v>
       </c>
-      <c r="U50" s="119"/>
+      <c r="U50" s="154"/>
       <c r="W50" s="115" t="s">
         <v>56</v>
       </c>
@@ -5066,22 +5496,22 @@
       <c r="I51" s="117" t="s">
         <v>197</v>
       </c>
-      <c r="K51" s="120" t="s">
+      <c r="K51" s="155" t="s">
         <v>180</v>
       </c>
-      <c r="L51" s="121"/>
-      <c r="N51" s="120" t="s">
+      <c r="L51" s="156"/>
+      <c r="N51" s="155" t="s">
         <v>180</v>
       </c>
-      <c r="O51" s="121"/>
-      <c r="Q51" s="120" t="s">
+      <c r="O51" s="156"/>
+      <c r="Q51" s="155" t="s">
         <v>180</v>
       </c>
-      <c r="R51" s="121"/>
-      <c r="T51" s="120" t="s">
+      <c r="R51" s="156"/>
+      <c r="T51" s="155" t="s">
         <v>180</v>
       </c>
-      <c r="U51" s="121"/>
+      <c r="U51" s="156"/>
       <c r="W51" s="117" t="s">
         <v>234</v>
       </c>
@@ -5102,49 +5532,2529 @@
       </c>
     </row>
     <row r="52" spans="2:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="126" t="s">
+      <c r="B52" s="143" t="s">
         <v>173</v>
       </c>
-      <c r="C52" s="127"/>
-      <c r="E52" s="126" t="s">
+      <c r="C52" s="144"/>
+      <c r="E52" s="143" t="s">
         <v>174</v>
       </c>
-      <c r="F52" s="127"/>
-      <c r="H52" s="126" t="s">
+      <c r="F52" s="144"/>
+      <c r="H52" s="143" t="s">
         <v>175</v>
       </c>
-      <c r="I52" s="127"/>
-      <c r="K52" s="122" t="s">
+      <c r="I52" s="144"/>
+      <c r="K52" s="145" t="s">
         <v>181</v>
       </c>
-      <c r="L52" s="123"/>
-      <c r="N52" s="122" t="s">
+      <c r="L52" s="146"/>
+      <c r="N52" s="145" t="s">
         <v>182</v>
       </c>
-      <c r="O52" s="123"/>
-      <c r="Q52" s="122" t="s">
+      <c r="O52" s="146"/>
+      <c r="Q52" s="145" t="s">
         <v>183</v>
       </c>
-      <c r="R52" s="123"/>
-      <c r="T52" s="122" t="s">
+      <c r="R52" s="146"/>
+      <c r="T52" s="145" t="s">
         <v>184</v>
       </c>
-      <c r="U52" s="123"/>
-      <c r="W52" s="126" t="s">
+      <c r="U52" s="146"/>
+      <c r="W52" s="143" t="s">
         <v>176</v>
       </c>
-      <c r="X52" s="127"/>
-      <c r="Z52" s="126" t="s">
+      <c r="X52" s="144"/>
+      <c r="Z52" s="143" t="s">
         <v>177</v>
       </c>
-      <c r="AA52" s="127"/>
-      <c r="AC52" s="126" t="s">
+      <c r="AA52" s="144"/>
+      <c r="AC52" s="143" t="s">
         <v>178</v>
       </c>
-      <c r="AD52" s="127"/>
+      <c r="AD52" s="144"/>
     </row>
   </sheetData>
   <mergeCells count="49">
+    <mergeCell ref="T52:U52"/>
+    <mergeCell ref="W52:X52"/>
+    <mergeCell ref="Z52:AA52"/>
+    <mergeCell ref="AC52:AD52"/>
+    <mergeCell ref="K51:L51"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="Q51:R51"/>
+    <mergeCell ref="T51:U51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="E52:F52"/>
+    <mergeCell ref="H52:I52"/>
+    <mergeCell ref="K52:L52"/>
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="Q52:R52"/>
+    <mergeCell ref="K49:L49"/>
+    <mergeCell ref="N49:O49"/>
+    <mergeCell ref="Q49:R49"/>
+    <mergeCell ref="T49:U49"/>
+    <mergeCell ref="K50:L50"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="Q50:R50"/>
+    <mergeCell ref="T50:U50"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="Y26:Y29"/>
+    <mergeCell ref="AB26:AB29"/>
+    <mergeCell ref="B47:G47"/>
+    <mergeCell ref="K47:N47"/>
+    <mergeCell ref="W47:AB47"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="W15:AA15"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="W18:AA18"/>
+    <mergeCell ref="W19:AA19"/>
+    <mergeCell ref="G20:H23"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="O10:R10"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="X11:AA11"/>
+    <mergeCell ref="L12:T12"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="X13:AA13"/>
+    <mergeCell ref="Y1:AC2"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="O6:R6"/>
+    <mergeCell ref="V6:AA6"/>
+    <mergeCell ref="V8:AA8"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="O9:R9"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>
+  <pageSetup scale="57" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{639F2336-69B3-4605-B191-23BB70925903}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AD52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="118"/>
+    <col min="3" max="3" width="7.28515625" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" customWidth="1"/>
+    <col min="7" max="7" width="8" customWidth="1"/>
+    <col min="8" max="8" width="7.85546875" customWidth="1"/>
+    <col min="9" max="10" width="7.28515625" customWidth="1"/>
+    <col min="11" max="11" width="8.5703125" customWidth="1"/>
+    <col min="12" max="12" width="8.28515625" customWidth="1"/>
+    <col min="13" max="13" width="7.140625" customWidth="1"/>
+    <col min="14" max="14" width="8.140625" customWidth="1"/>
+    <col min="15" max="15" width="7.7109375" customWidth="1"/>
+    <col min="16" max="16" width="7.28515625" customWidth="1"/>
+    <col min="17" max="17" width="8.7109375" customWidth="1"/>
+    <col min="18" max="18" width="8.5703125" customWidth="1"/>
+    <col min="19" max="19" width="7.28515625" customWidth="1"/>
+    <col min="20" max="20" width="8" customWidth="1"/>
+    <col min="21" max="21" width="7.7109375" customWidth="1"/>
+    <col min="22" max="25" width="7.28515625" customWidth="1"/>
+    <col min="26" max="26" width="9.140625" customWidth="1"/>
+    <col min="27" max="27" width="8.7109375" customWidth="1"/>
+    <col min="28" max="28" width="7.28515625" customWidth="1"/>
+    <col min="30" max="30" width="7.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R1" s="112" t="s">
+        <v>84</v>
+      </c>
+      <c r="S1" s="31" t="s">
+        <v>88</v>
+      </c>
+      <c r="T1" s="31" t="s">
+        <v>88</v>
+      </c>
+      <c r="U1" s="31" t="s">
+        <v>88</v>
+      </c>
+      <c r="V1" s="31" t="s">
+        <v>88</v>
+      </c>
+      <c r="W1" s="31" t="s">
+        <v>88</v>
+      </c>
+      <c r="X1" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="Y1" s="131" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z1" s="131"/>
+      <c r="AA1" s="131"/>
+      <c r="AB1" s="131"/>
+      <c r="AC1" s="131"/>
+    </row>
+    <row r="2" spans="1:30" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D2" s="62" t="s">
+        <v>86</v>
+      </c>
+      <c r="R2" s="112" t="s">
+        <v>91</v>
+      </c>
+      <c r="S2" s="31" t="s">
+        <v>88</v>
+      </c>
+      <c r="T2" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="U2" s="31" t="s">
+        <v>88</v>
+      </c>
+      <c r="V2" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="W2" s="31" t="s">
+        <v>88</v>
+      </c>
+      <c r="X2" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y2" s="131"/>
+      <c r="Z2" s="131"/>
+      <c r="AA2" s="131"/>
+      <c r="AB2" s="131"/>
+      <c r="AC2" s="131"/>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="E3" s="63" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="K5" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="L5" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="N5" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="O5" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="P5" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q5" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="R5" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="S5" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="T5" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="U5" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="V5" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="W5" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="X5" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="Y5" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="Z5" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="AA5" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB5" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="61" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="119" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="133" t="s">
+        <v>94</v>
+      </c>
+      <c r="H6" s="134"/>
+      <c r="I6" s="135"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="133" t="s">
+        <v>94</v>
+      </c>
+      <c r="P6" s="134"/>
+      <c r="Q6" s="134"/>
+      <c r="R6" s="135"/>
+      <c r="S6" s="64" t="s">
+        <v>49</v>
+      </c>
+      <c r="T6" s="1"/>
+      <c r="U6" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="V6" s="136" t="s">
+        <v>94</v>
+      </c>
+      <c r="W6" s="136"/>
+      <c r="X6" s="136"/>
+      <c r="Y6" s="136"/>
+      <c r="Z6" s="136"/>
+      <c r="AA6" s="136"/>
+      <c r="AB6" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="AC6" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="119" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="120" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7" s="72" t="s">
+        <v>110</v>
+      </c>
+      <c r="H7" s="73" t="s">
+        <v>115</v>
+      </c>
+      <c r="I7" s="74" t="s">
+        <v>107</v>
+      </c>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="105" t="s">
+        <v>103</v>
+      </c>
+      <c r="P7" s="106" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q7" s="107" t="s">
+        <v>98</v>
+      </c>
+      <c r="R7" s="108" t="s">
+        <v>92</v>
+      </c>
+      <c r="S7" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="102" t="s">
+        <v>104</v>
+      </c>
+      <c r="W7" s="103" t="s">
+        <v>134</v>
+      </c>
+      <c r="X7" s="103" t="s">
+        <v>147</v>
+      </c>
+      <c r="Y7" s="103" t="s">
+        <v>108</v>
+      </c>
+      <c r="Z7" s="103" t="s">
+        <v>152</v>
+      </c>
+      <c r="AA7" s="104" t="s">
+        <v>153</v>
+      </c>
+      <c r="AB7" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC7" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="AD7" s="120" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="120" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" s="75" t="s">
+        <v>109</v>
+      </c>
+      <c r="H8" s="76" t="s">
+        <v>116</v>
+      </c>
+      <c r="I8" s="77" t="s">
+        <v>105</v>
+      </c>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="109" t="s">
+        <v>106</v>
+      </c>
+      <c r="P8" s="110" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q8" s="111" t="s">
+        <v>95</v>
+      </c>
+      <c r="R8" s="108" t="s">
+        <v>93</v>
+      </c>
+      <c r="S8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="T8" s="1"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="122" t="s">
+        <v>38</v>
+      </c>
+      <c r="W8" s="123"/>
+      <c r="X8" s="123"/>
+      <c r="Y8" s="123"/>
+      <c r="Z8" s="123"/>
+      <c r="AA8" s="124"/>
+      <c r="AB8" s="1"/>
+      <c r="AC8" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="AD8" s="120" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="120" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="128" t="s">
+        <v>94</v>
+      </c>
+      <c r="H9" s="129"/>
+      <c r="I9" s="130"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="128" t="s">
+        <v>94</v>
+      </c>
+      <c r="P9" s="129"/>
+      <c r="Q9" s="129"/>
+      <c r="R9" s="130"/>
+      <c r="S9" s="1"/>
+      <c r="T9" s="1"/>
+      <c r="U9" s="1"/>
+      <c r="V9" s="1"/>
+      <c r="W9" s="1"/>
+      <c r="X9" s="1"/>
+      <c r="Y9" s="1"/>
+      <c r="Z9" s="1"/>
+      <c r="AA9" s="1"/>
+      <c r="AB9" s="1"/>
+      <c r="AC9" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD9" s="120" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="120" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="122" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="123"/>
+      <c r="I10" s="124"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="P10" s="123"/>
+      <c r="Q10" s="123"/>
+      <c r="R10" s="124"/>
+      <c r="S10" s="1"/>
+      <c r="T10" s="1"/>
+      <c r="U10" s="1"/>
+      <c r="V10" s="1"/>
+      <c r="W10" s="1"/>
+      <c r="X10" s="1"/>
+      <c r="Y10" s="1"/>
+      <c r="Z10" s="1"/>
+      <c r="AA10" s="1"/>
+      <c r="AB10" s="1"/>
+      <c r="AC10" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="AD10" s="120" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="120" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="133" t="s">
+        <v>94</v>
+      </c>
+      <c r="E11" s="134"/>
+      <c r="F11" s="134"/>
+      <c r="G11" s="135"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="3"/>
+      <c r="R11" s="3"/>
+      <c r="S11" s="3"/>
+      <c r="T11" s="3"/>
+      <c r="U11" s="2"/>
+      <c r="V11" s="1"/>
+      <c r="W11" s="1"/>
+      <c r="X11" s="133" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y11" s="134"/>
+      <c r="Z11" s="134"/>
+      <c r="AA11" s="135"/>
+      <c r="AB11" s="1"/>
+      <c r="AC11" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="AD11" s="120" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="120" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="7"/>
+      <c r="D12" s="78" t="s">
+        <v>117</v>
+      </c>
+      <c r="E12" s="79" t="s">
+        <v>119</v>
+      </c>
+      <c r="F12" s="79" t="s">
+        <v>121</v>
+      </c>
+      <c r="G12" s="80" t="s">
+        <v>122</v>
+      </c>
+      <c r="H12" s="9"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="137" t="s">
+        <v>31</v>
+      </c>
+      <c r="M12" s="138"/>
+      <c r="N12" s="138"/>
+      <c r="O12" s="138"/>
+      <c r="P12" s="138"/>
+      <c r="Q12" s="138"/>
+      <c r="R12" s="138"/>
+      <c r="S12" s="138"/>
+      <c r="T12" s="139"/>
+      <c r="U12" s="5"/>
+      <c r="V12" s="1"/>
+      <c r="W12" s="1"/>
+      <c r="X12" s="78" t="s">
+        <v>127</v>
+      </c>
+      <c r="Y12" s="79" t="s">
+        <v>139</v>
+      </c>
+      <c r="Z12" s="79" t="s">
+        <v>141</v>
+      </c>
+      <c r="AA12" s="80" t="s">
+        <v>142</v>
+      </c>
+      <c r="AB12" s="1"/>
+      <c r="AC12" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="AD12" s="120" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="120" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="1"/>
+      <c r="D13" s="122" t="s">
+        <v>58</v>
+      </c>
+      <c r="E13" s="123"/>
+      <c r="F13" s="123"/>
+      <c r="G13" s="124"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="6"/>
+      <c r="U13" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V13" s="1"/>
+      <c r="W13" s="1"/>
+      <c r="X13" s="122" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y13" s="123"/>
+      <c r="Z13" s="123"/>
+      <c r="AA13" s="124"/>
+      <c r="AB13" s="1"/>
+      <c r="AC13" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="AD13" s="120" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="120" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="133" t="s">
+        <v>94</v>
+      </c>
+      <c r="E14" s="134"/>
+      <c r="F14" s="134"/>
+      <c r="G14" s="135"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="69"/>
+      <c r="L14" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
+      <c r="R14" s="8"/>
+      <c r="S14" s="8"/>
+      <c r="T14" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="U14" s="99" t="s">
+        <v>154</v>
+      </c>
+      <c r="V14" s="9"/>
+      <c r="W14" s="1"/>
+      <c r="X14" s="1"/>
+      <c r="Y14" s="1"/>
+      <c r="Z14" s="1"/>
+      <c r="AA14" s="1"/>
+      <c r="AB14" s="1"/>
+      <c r="AC14" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="AD14" s="120" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="120" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="81" t="s">
+        <v>120</v>
+      </c>
+      <c r="E15" s="82" t="s">
+        <v>128</v>
+      </c>
+      <c r="F15" s="82" t="s">
+        <v>129</v>
+      </c>
+      <c r="G15" s="83" t="s">
+        <v>131</v>
+      </c>
+      <c r="H15" s="9"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="70"/>
+      <c r="L15" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="M15" s="11"/>
+      <c r="N15" s="11"/>
+      <c r="O15" s="11"/>
+      <c r="P15" s="11"/>
+      <c r="Q15" s="11"/>
+      <c r="R15" s="11"/>
+      <c r="S15" s="11"/>
+      <c r="T15" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U15" s="100"/>
+      <c r="V15" s="9"/>
+      <c r="W15" s="133" t="s">
+        <v>94</v>
+      </c>
+      <c r="X15" s="134"/>
+      <c r="Y15" s="134"/>
+      <c r="Z15" s="134"/>
+      <c r="AA15" s="135"/>
+      <c r="AB15" s="1"/>
+      <c r="AC15" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD15" s="120" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="120" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="81" t="s">
+        <v>135</v>
+      </c>
+      <c r="E16" s="82" t="s">
+        <v>136</v>
+      </c>
+      <c r="F16" s="83" t="s">
+        <v>145</v>
+      </c>
+      <c r="G16" s="65" t="s">
+        <v>55</v>
+      </c>
+      <c r="H16" s="9"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="70"/>
+      <c r="L16" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="M16" s="14"/>
+      <c r="N16" s="14"/>
+      <c r="O16" s="14"/>
+      <c r="P16" s="14"/>
+      <c r="Q16" s="14"/>
+      <c r="R16" s="14"/>
+      <c r="S16" s="14"/>
+      <c r="T16" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="U16" s="100"/>
+      <c r="V16" s="24"/>
+      <c r="W16" s="93" t="s">
+        <v>206</v>
+      </c>
+      <c r="X16" s="94" t="s">
+        <v>200</v>
+      </c>
+      <c r="Y16" s="94" t="s">
+        <v>222</v>
+      </c>
+      <c r="Z16" s="94" t="s">
+        <v>220</v>
+      </c>
+      <c r="AA16" s="95" t="s">
+        <v>151</v>
+      </c>
+      <c r="AB16" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="AC16" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="AD16" s="120" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="120" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="1"/>
+      <c r="D17" s="125" t="s">
+        <v>94</v>
+      </c>
+      <c r="E17" s="126"/>
+      <c r="F17" s="127"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="70"/>
+      <c r="L17" s="13">
+        <v>4</v>
+      </c>
+      <c r="M17" s="14"/>
+      <c r="N17" s="14"/>
+      <c r="O17" s="14"/>
+      <c r="P17" s="14"/>
+      <c r="Q17" s="14"/>
+      <c r="R17" s="14"/>
+      <c r="S17" s="14"/>
+      <c r="T17" s="15">
+        <v>1</v>
+      </c>
+      <c r="U17" s="100"/>
+      <c r="V17" s="24"/>
+      <c r="W17" s="96" t="s">
+        <v>207</v>
+      </c>
+      <c r="X17" s="97" t="s">
+        <v>205</v>
+      </c>
+      <c r="Y17" s="97" t="s">
+        <v>223</v>
+      </c>
+      <c r="Z17" s="97" t="s">
+        <v>221</v>
+      </c>
+      <c r="AA17" s="98" t="s">
+        <v>150</v>
+      </c>
+      <c r="AB17" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC17" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD17" s="120" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="120" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="70"/>
+      <c r="L18" s="13">
+        <v>5</v>
+      </c>
+      <c r="M18" s="14"/>
+      <c r="N18" s="14"/>
+      <c r="O18" s="14"/>
+      <c r="P18" s="14"/>
+      <c r="Q18" s="14"/>
+      <c r="R18" s="14"/>
+      <c r="S18" s="14"/>
+      <c r="T18" s="15">
+        <v>2</v>
+      </c>
+      <c r="U18" s="100"/>
+      <c r="V18" s="9"/>
+      <c r="W18" s="128" t="s">
+        <v>94</v>
+      </c>
+      <c r="X18" s="129"/>
+      <c r="Y18" s="129"/>
+      <c r="Z18" s="129"/>
+      <c r="AA18" s="130"/>
+      <c r="AB18" s="1"/>
+      <c r="AC18" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="AD18" s="120" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="120" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="67" t="s">
+        <v>96</v>
+      </c>
+      <c r="G19" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="H19" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="I19" s="67" t="s">
+        <v>97</v>
+      </c>
+      <c r="J19" s="24"/>
+      <c r="K19" s="70"/>
+      <c r="L19" s="13">
+        <v>6</v>
+      </c>
+      <c r="M19" s="14"/>
+      <c r="N19" s="14"/>
+      <c r="O19" s="14"/>
+      <c r="P19" s="14"/>
+      <c r="Q19" s="14"/>
+      <c r="R19" s="14"/>
+      <c r="S19" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="T19" s="15">
+        <v>42</v>
+      </c>
+      <c r="U19" s="100" t="s">
+        <v>202</v>
+      </c>
+      <c r="V19" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="W19" s="122" t="s">
+        <v>61</v>
+      </c>
+      <c r="X19" s="123"/>
+      <c r="Y19" s="123"/>
+      <c r="Z19" s="123"/>
+      <c r="AA19" s="124"/>
+      <c r="AB19" s="1"/>
+      <c r="AC19" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="AD19" s="120" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="120" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="113"/>
+      <c r="G20" s="140" t="s">
+        <v>50</v>
+      </c>
+      <c r="H20" s="140"/>
+      <c r="I20" s="114"/>
+      <c r="J20" s="24" t="s">
+        <v>201</v>
+      </c>
+      <c r="K20" s="70" t="s">
+        <v>216</v>
+      </c>
+      <c r="L20" s="13">
+        <v>7</v>
+      </c>
+      <c r="M20" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="N20" s="14"/>
+      <c r="O20" s="14"/>
+      <c r="P20" s="14"/>
+      <c r="Q20" s="14"/>
+      <c r="R20" s="14"/>
+      <c r="S20" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="T20" s="15">
+        <v>41</v>
+      </c>
+      <c r="U20" s="100" t="s">
+        <v>211</v>
+      </c>
+      <c r="V20" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="W20" s="1"/>
+      <c r="X20" s="1"/>
+      <c r="Y20" s="1"/>
+      <c r="Z20" s="1"/>
+      <c r="AA20" s="1"/>
+      <c r="AB20" s="1"/>
+      <c r="AC20" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="AD20" s="120" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="120" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" s="84" t="s">
+        <v>208</v>
+      </c>
+      <c r="E21" s="7"/>
+      <c r="F21" s="113"/>
+      <c r="G21" s="141"/>
+      <c r="H21" s="141"/>
+      <c r="I21" s="114"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="70"/>
+      <c r="L21" s="13">
+        <v>15</v>
+      </c>
+      <c r="M21" s="14"/>
+      <c r="N21" s="14"/>
+      <c r="O21" s="14"/>
+      <c r="P21" s="14"/>
+      <c r="Q21" s="14"/>
+      <c r="R21" s="14"/>
+      <c r="S21" s="14"/>
+      <c r="T21" s="15">
+        <v>40</v>
+      </c>
+      <c r="U21" s="100"/>
+      <c r="V21" s="9"/>
+      <c r="W21" s="1"/>
+      <c r="X21" s="1"/>
+      <c r="Y21" s="1"/>
+      <c r="Z21" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA21" s="84" t="s">
+        <v>224</v>
+      </c>
+      <c r="AB21" s="1"/>
+      <c r="AC21" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD21" s="120" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="120" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D22" s="85" t="s">
+        <v>209</v>
+      </c>
+      <c r="E22" s="7"/>
+      <c r="F22" s="113"/>
+      <c r="G22" s="141"/>
+      <c r="H22" s="141"/>
+      <c r="I22" s="114"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="70"/>
+      <c r="L22" s="13">
+        <v>16</v>
+      </c>
+      <c r="M22" s="14"/>
+      <c r="N22" s="14"/>
+      <c r="O22" s="14"/>
+      <c r="P22" s="14"/>
+      <c r="Q22" s="14"/>
+      <c r="R22" s="14"/>
+      <c r="S22" s="14"/>
+      <c r="T22" s="15">
+        <v>39</v>
+      </c>
+      <c r="U22" s="100"/>
+      <c r="V22" s="9"/>
+      <c r="W22" s="1"/>
+      <c r="X22" s="1"/>
+      <c r="Y22" s="1"/>
+      <c r="Z22" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA22" s="85" t="s">
+        <v>225</v>
+      </c>
+      <c r="AB22" s="1"/>
+      <c r="AC22" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD22" s="120" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="120" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D23" s="86" t="s">
+        <v>210</v>
+      </c>
+      <c r="E23" s="7"/>
+      <c r="F23" s="113"/>
+      <c r="G23" s="142"/>
+      <c r="H23" s="142"/>
+      <c r="I23" s="114"/>
+      <c r="J23" s="24"/>
+      <c r="K23" s="70"/>
+      <c r="L23" s="13">
+        <v>17</v>
+      </c>
+      <c r="M23" s="14"/>
+      <c r="N23" s="14"/>
+      <c r="O23" s="14"/>
+      <c r="P23" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q23" s="14"/>
+      <c r="R23" s="14"/>
+      <c r="S23" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="T23" s="15">
+        <v>38</v>
+      </c>
+      <c r="U23" s="100" t="s">
+        <v>227</v>
+      </c>
+      <c r="V23" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="W23" s="1"/>
+      <c r="X23" s="1"/>
+      <c r="Y23" s="1"/>
+      <c r="Z23" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="AA23" s="86" t="s">
+        <v>226</v>
+      </c>
+      <c r="AB23" s="1"/>
+      <c r="AC23" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD23" s="120" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="120" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E24" s="7"/>
+      <c r="F24" s="67" t="s">
+        <v>132</v>
+      </c>
+      <c r="G24" s="27" t="s">
+        <v>53</v>
+      </c>
+      <c r="H24" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="I24" s="67" t="s">
+        <v>133</v>
+      </c>
+      <c r="J24" s="24"/>
+      <c r="K24" s="70"/>
+      <c r="L24" s="13">
+        <v>18</v>
+      </c>
+      <c r="M24" s="14"/>
+      <c r="N24" s="14"/>
+      <c r="O24" s="14"/>
+      <c r="P24" s="14"/>
+      <c r="Q24" s="14"/>
+      <c r="R24" s="14"/>
+      <c r="S24" s="14"/>
+      <c r="T24" s="15">
+        <v>37</v>
+      </c>
+      <c r="U24" s="100"/>
+      <c r="V24" s="9"/>
+      <c r="W24" s="1"/>
+      <c r="X24" s="1"/>
+      <c r="Y24" s="1"/>
+      <c r="Z24" s="1"/>
+      <c r="AA24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB24" s="1"/>
+      <c r="AC24" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD24" s="120" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="120" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="1"/>
+      <c r="D25" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="E25" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="70"/>
+      <c r="L25" s="13">
+        <v>8</v>
+      </c>
+      <c r="M25" s="14"/>
+      <c r="N25" s="14"/>
+      <c r="O25" s="14"/>
+      <c r="P25" s="14"/>
+      <c r="Q25" s="14"/>
+      <c r="R25" s="14"/>
+      <c r="S25" s="14"/>
+      <c r="T25" s="15">
+        <v>36</v>
+      </c>
+      <c r="U25" s="100"/>
+      <c r="V25" s="9"/>
+      <c r="W25" s="1"/>
+      <c r="X25" s="1"/>
+      <c r="Y25" s="1"/>
+      <c r="Z25" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA25" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB25" s="1"/>
+      <c r="AC25" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD25" s="120" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="120" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="147" t="s">
+        <v>94</v>
+      </c>
+      <c r="D26" s="87" t="s">
+        <v>167</v>
+      </c>
+      <c r="E26" s="88" t="s">
+        <v>168</v>
+      </c>
+      <c r="F26" s="150" t="s">
+        <v>94</v>
+      </c>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="70"/>
+      <c r="L26" s="13">
+        <v>3</v>
+      </c>
+      <c r="M26" s="14"/>
+      <c r="N26" s="14"/>
+      <c r="O26" s="14"/>
+      <c r="P26" s="14"/>
+      <c r="Q26" s="14"/>
+      <c r="R26" s="14"/>
+      <c r="S26" s="14"/>
+      <c r="T26" s="15">
+        <v>35</v>
+      </c>
+      <c r="U26" s="100"/>
+      <c r="V26" s="9"/>
+      <c r="W26" s="1"/>
+      <c r="X26" s="1"/>
+      <c r="Y26" s="147" t="s">
+        <v>94</v>
+      </c>
+      <c r="Z26" s="87" t="s">
+        <v>172</v>
+      </c>
+      <c r="AA26" s="88" t="s">
+        <v>171</v>
+      </c>
+      <c r="AB26" s="150" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC26" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="AD26" s="120" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="120" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="148"/>
+      <c r="D27" s="89" t="s">
+        <v>190</v>
+      </c>
+      <c r="E27" s="90" t="s">
+        <v>189</v>
+      </c>
+      <c r="F27" s="151"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="70"/>
+      <c r="L27" s="13">
+        <v>46</v>
+      </c>
+      <c r="M27" s="14"/>
+      <c r="N27" s="14"/>
+      <c r="O27" s="14"/>
+      <c r="P27" s="14"/>
+      <c r="Q27" s="14"/>
+      <c r="R27" s="14"/>
+      <c r="S27" s="14"/>
+      <c r="T27" s="15">
+        <v>0</v>
+      </c>
+      <c r="U27" s="100"/>
+      <c r="V27" s="9"/>
+      <c r="W27" s="1"/>
+      <c r="X27" s="1"/>
+      <c r="Y27" s="148"/>
+      <c r="Z27" s="89" t="s">
+        <v>230</v>
+      </c>
+      <c r="AA27" s="90" t="s">
+        <v>231</v>
+      </c>
+      <c r="AB27" s="151"/>
+      <c r="AC27" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="AD27" s="120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="120" t="s">
+        <v>8</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="148"/>
+      <c r="D28" s="89" t="s">
+        <v>191</v>
+      </c>
+      <c r="E28" s="90" t="s">
+        <v>188</v>
+      </c>
+      <c r="F28" s="151"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="70"/>
+      <c r="L28" s="13">
+        <v>9</v>
+      </c>
+      <c r="M28" s="14"/>
+      <c r="N28" s="14"/>
+      <c r="O28" s="14"/>
+      <c r="P28" s="14"/>
+      <c r="Q28" s="14"/>
+      <c r="R28" s="14"/>
+      <c r="S28" s="14"/>
+      <c r="T28" s="15">
+        <v>45</v>
+      </c>
+      <c r="U28" s="100"/>
+      <c r="V28" s="9"/>
+      <c r="W28" s="1"/>
+      <c r="X28" s="1"/>
+      <c r="Y28" s="148"/>
+      <c r="Z28" s="89" t="s">
+        <v>229</v>
+      </c>
+      <c r="AA28" s="90" t="s">
+        <v>232</v>
+      </c>
+      <c r="AB28" s="151"/>
+      <c r="AC28" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="AD28" s="120" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="120" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C29" s="149"/>
+      <c r="D29" s="91" t="s">
+        <v>186</v>
+      </c>
+      <c r="E29" s="92" t="s">
+        <v>187</v>
+      </c>
+      <c r="F29" s="152"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="K29" s="70" t="s">
+        <v>161</v>
+      </c>
+      <c r="L29" s="13">
+        <v>10</v>
+      </c>
+      <c r="M29" s="14"/>
+      <c r="N29" s="14"/>
+      <c r="O29" s="14"/>
+      <c r="P29" s="14"/>
+      <c r="Q29" s="14"/>
+      <c r="R29" s="14"/>
+      <c r="S29" s="14"/>
+      <c r="T29" s="15">
+        <v>48</v>
+      </c>
+      <c r="U29" s="100"/>
+      <c r="V29" s="9"/>
+      <c r="W29" s="1"/>
+      <c r="X29" s="1"/>
+      <c r="Y29" s="149"/>
+      <c r="Z29" s="91" t="s">
+        <v>228</v>
+      </c>
+      <c r="AA29" s="92" t="s">
+        <v>233</v>
+      </c>
+      <c r="AB29" s="152"/>
+      <c r="AC29" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="AD29" s="120" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="120" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="1"/>
+      <c r="D30" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="E30" s="17"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="K30" s="70" t="s">
+        <v>162</v>
+      </c>
+      <c r="L30" s="13">
+        <v>11</v>
+      </c>
+      <c r="M30" s="14"/>
+      <c r="N30" s="14"/>
+      <c r="O30" s="14"/>
+      <c r="P30" s="14"/>
+      <c r="Q30" s="14"/>
+      <c r="R30" s="14"/>
+      <c r="S30" s="14"/>
+      <c r="T30" s="15">
+        <v>47</v>
+      </c>
+      <c r="U30" s="100"/>
+      <c r="V30" s="9"/>
+      <c r="W30" s="1"/>
+      <c r="X30" s="1"/>
+      <c r="Y30" s="1"/>
+      <c r="Z30" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA30" s="17"/>
+      <c r="AB30" s="1"/>
+      <c r="AC30" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="AD30" s="120" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="120" t="s">
+        <v>5</v>
+      </c>
+      <c r="B31" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="K31" s="70" t="s">
+        <v>157</v>
+      </c>
+      <c r="L31" s="13">
+        <v>12</v>
+      </c>
+      <c r="M31" s="14"/>
+      <c r="N31" s="14"/>
+      <c r="O31" s="14"/>
+      <c r="P31" s="14"/>
+      <c r="Q31" s="14"/>
+      <c r="R31" s="14"/>
+      <c r="S31" s="14"/>
+      <c r="T31" s="15">
+        <v>21</v>
+      </c>
+      <c r="U31" s="100"/>
+      <c r="V31" s="9"/>
+      <c r="W31" s="1"/>
+      <c r="X31" s="1"/>
+      <c r="Y31" s="1"/>
+      <c r="Z31" s="1"/>
+      <c r="AA31" s="1"/>
+      <c r="AB31" s="1"/>
+      <c r="AC31" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="AD31" s="120" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="120" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D32" s="84" t="s">
+        <v>203</v>
+      </c>
+      <c r="E32" s="1"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="K32" s="70" t="s">
+        <v>158</v>
+      </c>
+      <c r="L32" s="13">
+        <v>13</v>
+      </c>
+      <c r="M32" s="14"/>
+      <c r="N32" s="14"/>
+      <c r="O32" s="14"/>
+      <c r="P32" s="14"/>
+      <c r="Q32" s="14"/>
+      <c r="R32" s="14"/>
+      <c r="S32" s="14"/>
+      <c r="T32" s="15">
+        <v>20</v>
+      </c>
+      <c r="U32" s="100"/>
+      <c r="V32" s="9"/>
+      <c r="W32" s="1"/>
+      <c r="X32" s="1"/>
+      <c r="Y32" s="1"/>
+      <c r="Z32" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA32" s="84" t="s">
+        <v>218</v>
+      </c>
+      <c r="AB32" s="1"/>
+      <c r="AC32" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="AD32" s="120" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="120" t="s">
+        <v>3</v>
+      </c>
+      <c r="B33" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D33" s="85" t="s">
+        <v>204</v>
+      </c>
+      <c r="E33" s="1"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="7"/>
+      <c r="K33" s="70"/>
+      <c r="L33" s="13">
+        <v>14</v>
+      </c>
+      <c r="M33" s="14"/>
+      <c r="N33" s="14"/>
+      <c r="O33" s="14"/>
+      <c r="P33" s="14"/>
+      <c r="Q33" s="14"/>
+      <c r="R33" s="14"/>
+      <c r="S33" s="14"/>
+      <c r="T33" s="15">
+        <v>19</v>
+      </c>
+      <c r="U33" s="100"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="1"/>
+      <c r="X33" s="1"/>
+      <c r="Y33" s="1"/>
+      <c r="Z33" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA33" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="AB33" s="1"/>
+      <c r="AC33" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="AD33" s="120" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="120" t="s">
+        <v>2</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D34" s="86" t="s">
+        <v>199</v>
+      </c>
+      <c r="E34" s="1"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="7"/>
+      <c r="K34" s="70" t="s">
+        <v>130</v>
+      </c>
+      <c r="L34" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="M34" s="19"/>
+      <c r="N34" s="19"/>
+      <c r="O34" s="19"/>
+      <c r="P34" s="19"/>
+      <c r="Q34" s="19"/>
+      <c r="R34" s="19"/>
+      <c r="S34" s="19"/>
+      <c r="T34" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="U34" s="100"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="1"/>
+      <c r="X34" s="1"/>
+      <c r="Y34" s="1"/>
+      <c r="Z34" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="AA34" s="86" t="s">
+        <v>217</v>
+      </c>
+      <c r="AB34" s="1"/>
+      <c r="AC34" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD34" s="120" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="120" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C35" s="1"/>
+      <c r="D35" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="7"/>
+      <c r="K35" s="71" t="s">
+        <v>146</v>
+      </c>
+      <c r="L35" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="M35" s="21"/>
+      <c r="N35" s="21"/>
+      <c r="O35" s="21"/>
+      <c r="P35" s="21"/>
+      <c r="Q35" s="21"/>
+      <c r="R35" s="21"/>
+      <c r="S35" s="21"/>
+      <c r="T35" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="U35" s="101"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="1"/>
+      <c r="X35" s="1"/>
+      <c r="Y35" s="1"/>
+      <c r="Z35" s="1"/>
+      <c r="AA35" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB35" s="1"/>
+      <c r="AC35" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD35" s="120" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:30" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="121" t="s">
+        <v>0</v>
+      </c>
+      <c r="B36" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="L36" s="17"/>
+      <c r="M36" s="17"/>
+      <c r="N36" s="17"/>
+      <c r="O36" s="17"/>
+      <c r="P36" s="17"/>
+      <c r="Q36" s="17"/>
+      <c r="R36" s="17"/>
+      <c r="S36" s="17"/>
+      <c r="T36" s="17"/>
+      <c r="U36" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="V36" s="1"/>
+      <c r="W36" s="1"/>
+      <c r="X36" s="1"/>
+      <c r="Y36" s="1"/>
+      <c r="Z36" s="1"/>
+      <c r="AA36" s="1"/>
+      <c r="AB36" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="AC36" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="AD36" s="121" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="B37" s="23"/>
+      <c r="C37" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="E37" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="F37" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="G37" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="H37" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="I37" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="J37" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="K37" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="L37" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="M37" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="N37" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="O37" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="P37" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q37" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="R37" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="S37" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="T37" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="U37" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="V37" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="W37" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="X37" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="Y37" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="Z37" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="AA37" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB37" s="22" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="32"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="33"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="34"/>
+      <c r="G40" s="35"/>
+      <c r="K40" s="49"/>
+      <c r="L40" s="59"/>
+      <c r="M40" s="59"/>
+      <c r="N40" s="50"/>
+      <c r="W40" s="32"/>
+      <c r="X40" s="33"/>
+      <c r="Y40" s="33"/>
+      <c r="Z40" s="33"/>
+      <c r="AA40" s="34"/>
+      <c r="AB40" s="35"/>
+    </row>
+    <row r="41" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="36"/>
+      <c r="C41" s="66" t="s">
+        <v>112</v>
+      </c>
+      <c r="D41" s="66" t="s">
+        <v>111</v>
+      </c>
+      <c r="E41" s="66" t="s">
+        <v>166</v>
+      </c>
+      <c r="F41" s="66" t="s">
+        <v>165</v>
+      </c>
+      <c r="G41" s="37"/>
+      <c r="K41" s="56" t="s">
+        <v>83</v>
+      </c>
+      <c r="L41" s="67" t="s">
+        <v>101</v>
+      </c>
+      <c r="M41" s="67" t="s">
+        <v>102</v>
+      </c>
+      <c r="N41" s="58"/>
+      <c r="W41" s="36"/>
+      <c r="X41" s="66" t="s">
+        <v>113</v>
+      </c>
+      <c r="Y41" s="66" t="s">
+        <v>114</v>
+      </c>
+      <c r="Z41" s="66" t="s">
+        <v>169</v>
+      </c>
+      <c r="AA41" s="66" t="s">
+        <v>170</v>
+      </c>
+      <c r="AB41" s="37"/>
+    </row>
+    <row r="42" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="B42" s="38"/>
+      <c r="C42" s="48" t="s">
+        <v>68</v>
+      </c>
+      <c r="D42" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="E42" s="48" t="s">
+        <v>70</v>
+      </c>
+      <c r="F42" s="48" t="s">
+        <v>71</v>
+      </c>
+      <c r="G42" s="39"/>
+      <c r="K42" s="51"/>
+      <c r="L42" s="60" t="s">
+        <v>57</v>
+      </c>
+      <c r="M42" s="60" t="s">
+        <v>56</v>
+      </c>
+      <c r="N42" s="53"/>
+      <c r="W42" s="38"/>
+      <c r="X42" s="48" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y42" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="Z42" s="48" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA42" s="48" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB42" s="39"/>
+    </row>
+    <row r="43" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="38"/>
+      <c r="C43" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="D43" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="E43" s="40" t="s">
+        <v>75</v>
+      </c>
+      <c r="F43" s="40" t="s">
+        <v>74</v>
+      </c>
+      <c r="G43" s="39"/>
+      <c r="K43" s="51"/>
+      <c r="L43" s="52"/>
+      <c r="M43" s="52"/>
+      <c r="N43" s="53"/>
+      <c r="W43" s="38"/>
+      <c r="X43" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="Y43" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="Z43" s="40" t="s">
+        <v>75</v>
+      </c>
+      <c r="AA43" s="40" t="s">
+        <v>74</v>
+      </c>
+      <c r="AB43" s="39"/>
+    </row>
+    <row r="44" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B44" s="36">
+        <v>7</v>
+      </c>
+      <c r="C44" s="66" t="s">
+        <v>118</v>
+      </c>
+      <c r="D44" s="68" t="s">
+        <v>123</v>
+      </c>
+      <c r="E44" s="66" t="s">
+        <v>125</v>
+      </c>
+      <c r="F44" s="66" t="s">
+        <v>156</v>
+      </c>
+      <c r="G44" s="42">
+        <v>1</v>
+      </c>
+      <c r="K44" s="51"/>
+      <c r="L44" s="57"/>
+      <c r="M44" s="57"/>
+      <c r="N44" s="53"/>
+      <c r="W44" s="36">
+        <v>7</v>
+      </c>
+      <c r="X44" s="66" t="s">
+        <v>140</v>
+      </c>
+      <c r="Y44" s="68" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z44" s="66" t="s">
+        <v>143</v>
+      </c>
+      <c r="AA44" s="66" t="s">
+        <v>163</v>
+      </c>
+      <c r="AB44" s="42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B45" s="36">
+        <v>8</v>
+      </c>
+      <c r="C45" s="66" t="s">
+        <v>137</v>
+      </c>
+      <c r="D45" s="68" t="s">
+        <v>124</v>
+      </c>
+      <c r="E45" s="66" t="s">
+        <v>126</v>
+      </c>
+      <c r="F45" s="66" t="s">
+        <v>155</v>
+      </c>
+      <c r="G45" s="39">
+        <v>2</v>
+      </c>
+      <c r="K45" s="56" t="s">
+        <v>82</v>
+      </c>
+      <c r="L45" s="67" t="s">
+        <v>148</v>
+      </c>
+      <c r="M45" s="67" t="s">
+        <v>149</v>
+      </c>
+      <c r="N45" s="58"/>
+      <c r="W45" s="36">
+        <v>8</v>
+      </c>
+      <c r="X45" s="66" t="s">
+        <v>138</v>
+      </c>
+      <c r="Y45" s="68" t="s">
+        <v>124</v>
+      </c>
+      <c r="Z45" s="66" t="s">
+        <v>144</v>
+      </c>
+      <c r="AA45" s="66" t="s">
+        <v>164</v>
+      </c>
+      <c r="AB45" s="39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="43"/>
+      <c r="C46" s="44" t="s">
+        <v>43</v>
+      </c>
+      <c r="D46" s="45" t="s">
+        <v>77</v>
+      </c>
+      <c r="E46" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="F46" s="46" t="s">
+        <v>73</v>
+      </c>
+      <c r="G46" s="47"/>
+      <c r="K46" s="54"/>
+      <c r="L46" s="60" t="s">
+        <v>57</v>
+      </c>
+      <c r="M46" s="60" t="s">
+        <v>56</v>
+      </c>
+      <c r="N46" s="55"/>
+      <c r="W46" s="43"/>
+      <c r="X46" s="44" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y46" s="45" t="s">
+        <v>77</v>
+      </c>
+      <c r="Z46" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="AA46" s="46" t="s">
+        <v>73</v>
+      </c>
+      <c r="AB46" s="47"/>
+    </row>
+    <row r="47" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="B47" s="132" t="s">
+        <v>79</v>
+      </c>
+      <c r="C47" s="132"/>
+      <c r="D47" s="132"/>
+      <c r="E47" s="132"/>
+      <c r="F47" s="132"/>
+      <c r="G47" s="132"/>
+      <c r="K47" s="132" t="s">
+        <v>81</v>
+      </c>
+      <c r="L47" s="132"/>
+      <c r="M47" s="132"/>
+      <c r="N47" s="132"/>
+      <c r="W47" s="132" t="s">
+        <v>80</v>
+      </c>
+      <c r="X47" s="132"/>
+      <c r="Y47" s="132"/>
+      <c r="Z47" s="132"/>
+      <c r="AA47" s="132"/>
+      <c r="AB47" s="132"/>
+    </row>
+    <row r="48" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="49" spans="2:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K49" s="157" t="s">
+        <v>185</v>
+      </c>
+      <c r="L49" s="158"/>
+      <c r="N49" s="157" t="s">
+        <v>198</v>
+      </c>
+      <c r="O49" s="158"/>
+      <c r="Q49" s="157" t="s">
+        <v>240</v>
+      </c>
+      <c r="R49" s="158"/>
+      <c r="T49" s="157" t="s">
+        <v>241</v>
+      </c>
+      <c r="U49" s="158"/>
+    </row>
+    <row r="50" spans="2:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B50" s="115" t="s">
+        <v>56</v>
+      </c>
+      <c r="C50" s="116" t="s">
+        <v>57</v>
+      </c>
+      <c r="E50" s="115" t="s">
+        <v>56</v>
+      </c>
+      <c r="F50" s="116" t="s">
+        <v>57</v>
+      </c>
+      <c r="H50" s="115" t="s">
+        <v>56</v>
+      </c>
+      <c r="I50" s="116" t="s">
+        <v>57</v>
+      </c>
+      <c r="K50" s="153" t="s">
+        <v>179</v>
+      </c>
+      <c r="L50" s="154"/>
+      <c r="N50" s="153" t="s">
+        <v>179</v>
+      </c>
+      <c r="O50" s="154"/>
+      <c r="Q50" s="153" t="s">
+        <v>179</v>
+      </c>
+      <c r="R50" s="154"/>
+      <c r="T50" s="153" t="s">
+        <v>179</v>
+      </c>
+      <c r="U50" s="154"/>
+      <c r="W50" s="115" t="s">
+        <v>56</v>
+      </c>
+      <c r="X50" s="116" t="s">
+        <v>57</v>
+      </c>
+      <c r="Z50" s="115" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA50" s="116" t="s">
+        <v>57</v>
+      </c>
+      <c r="AC50" s="115" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD50" s="116" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="51" spans="2:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="117" t="s">
+        <v>192</v>
+      </c>
+      <c r="C51" s="117" t="s">
+        <v>193</v>
+      </c>
+      <c r="E51" s="117" t="s">
+        <v>194</v>
+      </c>
+      <c r="F51" s="117" t="s">
+        <v>195</v>
+      </c>
+      <c r="H51" s="117" t="s">
+        <v>196</v>
+      </c>
+      <c r="I51" s="117" t="s">
+        <v>197</v>
+      </c>
+      <c r="K51" s="155" t="s">
+        <v>180</v>
+      </c>
+      <c r="L51" s="156"/>
+      <c r="N51" s="155" t="s">
+        <v>180</v>
+      </c>
+      <c r="O51" s="156"/>
+      <c r="Q51" s="155" t="s">
+        <v>180</v>
+      </c>
+      <c r="R51" s="156"/>
+      <c r="T51" s="155" t="s">
+        <v>180</v>
+      </c>
+      <c r="U51" s="156"/>
+      <c r="W51" s="117" t="s">
+        <v>234</v>
+      </c>
+      <c r="X51" s="117" t="s">
+        <v>235</v>
+      </c>
+      <c r="Z51" s="117" t="s">
+        <v>236</v>
+      </c>
+      <c r="AA51" s="117" t="s">
+        <v>237</v>
+      </c>
+      <c r="AC51" s="117" t="s">
+        <v>238</v>
+      </c>
+      <c r="AD51" s="117" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="52" spans="2:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B52" s="143" t="s">
+        <v>173</v>
+      </c>
+      <c r="C52" s="144"/>
+      <c r="E52" s="143" t="s">
+        <v>174</v>
+      </c>
+      <c r="F52" s="144"/>
+      <c r="H52" s="143" t="s">
+        <v>175</v>
+      </c>
+      <c r="I52" s="144"/>
+      <c r="K52" s="145" t="s">
+        <v>181</v>
+      </c>
+      <c r="L52" s="146"/>
+      <c r="N52" s="145" t="s">
+        <v>182</v>
+      </c>
+      <c r="O52" s="146"/>
+      <c r="Q52" s="145" t="s">
+        <v>183</v>
+      </c>
+      <c r="R52" s="146"/>
+      <c r="T52" s="145" t="s">
+        <v>184</v>
+      </c>
+      <c r="U52" s="146"/>
+      <c r="W52" s="143" t="s">
+        <v>176</v>
+      </c>
+      <c r="X52" s="144"/>
+      <c r="Z52" s="143" t="s">
+        <v>177</v>
+      </c>
+      <c r="AA52" s="144"/>
+      <c r="AC52" s="143" t="s">
+        <v>178</v>
+      </c>
+      <c r="AD52" s="144"/>
+    </row>
+  </sheetData>
+  <mergeCells count="49">
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="Q50:R50"/>
+    <mergeCell ref="Q51:R51"/>
+    <mergeCell ref="Q52:R52"/>
+    <mergeCell ref="Q49:R49"/>
+    <mergeCell ref="T49:U49"/>
+    <mergeCell ref="K50:L50"/>
+    <mergeCell ref="K51:L51"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="AC52:AD52"/>
+    <mergeCell ref="K52:L52"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="AB26:AB29"/>
+    <mergeCell ref="Y26:Y29"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="E52:F52"/>
+    <mergeCell ref="H52:I52"/>
+    <mergeCell ref="W52:X52"/>
+    <mergeCell ref="Z52:AA52"/>
+    <mergeCell ref="T50:U50"/>
+    <mergeCell ref="T51:U51"/>
+    <mergeCell ref="T52:U52"/>
+    <mergeCell ref="K49:L49"/>
+    <mergeCell ref="N49:O49"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="O9:R9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="W15:AA15"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="X13:AA13"/>
     <mergeCell ref="W19:AA19"/>
     <mergeCell ref="D17:F17"/>
     <mergeCell ref="W18:AA18"/>
@@ -5161,39 +8071,6 @@
     <mergeCell ref="O10:R10"/>
     <mergeCell ref="G20:H23"/>
     <mergeCell ref="D13:G13"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="O9:R9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="W15:AA15"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="D14:G14"/>
-    <mergeCell ref="X13:AA13"/>
-    <mergeCell ref="AC52:AD52"/>
-    <mergeCell ref="K52:L52"/>
-    <mergeCell ref="C26:C29"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="AB26:AB29"/>
-    <mergeCell ref="Y26:Y29"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="E52:F52"/>
-    <mergeCell ref="H52:I52"/>
-    <mergeCell ref="W52:X52"/>
-    <mergeCell ref="Z52:AA52"/>
-    <mergeCell ref="T50:U50"/>
-    <mergeCell ref="T51:U51"/>
-    <mergeCell ref="T52:U52"/>
-    <mergeCell ref="K49:L49"/>
-    <mergeCell ref="N49:O49"/>
-    <mergeCell ref="Q49:R49"/>
-    <mergeCell ref="T49:U49"/>
-    <mergeCell ref="K50:L50"/>
-    <mergeCell ref="K51:L51"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:O52"/>
-    <mergeCell ref="Q50:R50"/>
-    <mergeCell ref="Q51:R51"/>
-    <mergeCell ref="Q52:R52"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>

</xml_diff>